<commit_message>
Fase C faerdig: valideringsscenarier for cat10-rest + cat12 (98/98 aktive kontroller); test-felt udledt i katalog/matrix
</commit_message>
<xml_diff>
--- a/docs/VAT-Analytics_Regel-sporbarhedsmatrix.xlsx
+++ b/docs/VAT-Analytics_Regel-sporbarhedsmatrix.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oversigt" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sporbarhedsmatrix" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kategorier" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Oversigt" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sporbarhedsmatrix" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Kategorier" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Oversigt'!$A$1:$B$1</definedName>
@@ -543,7 +543,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>0 / 103</t>
+          <t>98 / 103</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr"/>
@@ -757,7 +757,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr"/>
@@ -813,7 +813,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr"/>
@@ -869,7 +869,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr"/>
@@ -925,7 +925,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr"/>
@@ -981,7 +981,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr"/>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr"/>
@@ -1093,7 +1093,7 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr"/>
@@ -1149,7 +1149,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr"/>
@@ -1205,7 +1205,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr"/>
@@ -1261,7 +1261,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr"/>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr"/>
@@ -1373,7 +1373,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr"/>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr"/>
@@ -1485,7 +1485,7 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr"/>
@@ -1541,7 +1541,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr"/>
@@ -1597,7 +1597,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr"/>
@@ -1653,7 +1653,7 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr"/>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr"/>
@@ -1765,7 +1765,7 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr"/>
@@ -1821,7 +1821,7 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr"/>
@@ -1877,7 +1877,7 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr"/>
@@ -1933,7 +1933,7 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr"/>
@@ -1989,7 +1989,7 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr"/>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr"/>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr"/>
@@ -2157,7 +2157,7 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr"/>
@@ -2213,7 +2213,7 @@
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr"/>
@@ -2269,7 +2269,7 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr"/>
@@ -2325,7 +2325,7 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr"/>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr"/>
@@ -2437,7 +2437,7 @@
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr"/>
@@ -2493,7 +2493,7 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr"/>
@@ -2549,7 +2549,7 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr"/>
@@ -2605,7 +2605,7 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr"/>
@@ -2661,7 +2661,7 @@
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr"/>
@@ -2777,7 +2777,7 @@
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr"/>
@@ -2833,7 +2833,7 @@
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr"/>
@@ -2889,7 +2889,7 @@
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L41" s="2" t="inlineStr"/>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr"/>
@@ -3001,7 +3001,7 @@
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr"/>
@@ -3057,7 +3057,7 @@
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr"/>
@@ -3113,7 +3113,7 @@
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr"/>
@@ -3169,7 +3169,7 @@
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr"/>
@@ -3225,7 +3225,7 @@
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L47" s="2" t="inlineStr">
@@ -3285,7 +3285,7 @@
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr"/>
@@ -3341,7 +3341,7 @@
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L49" s="2" t="inlineStr"/>
@@ -3397,7 +3397,7 @@
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L50" s="2" t="inlineStr"/>
@@ -3453,7 +3453,7 @@
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L51" s="2" t="inlineStr"/>
@@ -3509,7 +3509,7 @@
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr"/>
@@ -3565,7 +3565,7 @@
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L53" s="2" t="inlineStr"/>
@@ -3621,7 +3621,7 @@
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L54" s="2" t="inlineStr"/>
@@ -3677,7 +3677,7 @@
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L55" s="2" t="inlineStr"/>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L56" s="2" t="inlineStr"/>
@@ -3789,7 +3789,7 @@
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L57" s="2" t="inlineStr"/>
@@ -3845,7 +3845,7 @@
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L58" s="2" t="inlineStr"/>
@@ -3901,7 +3901,7 @@
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L59" s="2" t="inlineStr"/>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L60" s="2" t="inlineStr"/>
@@ -4013,7 +4013,7 @@
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L61" s="2" t="inlineStr"/>
@@ -4069,7 +4069,7 @@
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L62" s="2" t="inlineStr"/>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L63" s="2" t="inlineStr"/>
@@ -4181,7 +4181,7 @@
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr"/>
@@ -4237,7 +4237,7 @@
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L65" s="2" t="inlineStr"/>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L66" s="2" t="inlineStr"/>
@@ -4349,7 +4349,7 @@
       </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L67" s="2" t="inlineStr"/>
@@ -4405,7 +4405,7 @@
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L68" s="2" t="inlineStr"/>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L69" s="2" t="inlineStr"/>
@@ -4517,7 +4517,7 @@
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L70" s="2" t="inlineStr"/>
@@ -4573,7 +4573,7 @@
       </c>
       <c r="K71" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L71" s="2" t="inlineStr"/>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L72" s="2" t="inlineStr"/>
@@ -4685,7 +4685,7 @@
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L73" s="2" t="inlineStr"/>
@@ -4741,7 +4741,7 @@
       </c>
       <c r="K74" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L74" s="2" t="inlineStr"/>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="K75" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L75" s="2" t="inlineStr"/>
@@ -4853,7 +4853,7 @@
       </c>
       <c r="K76" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L76" s="2" t="inlineStr"/>
@@ -4909,7 +4909,7 @@
       </c>
       <c r="K77" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L77" s="2" t="inlineStr"/>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="K78" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L78" s="2" t="inlineStr"/>
@@ -5021,7 +5021,7 @@
       </c>
       <c r="K79" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L79" s="2" t="inlineStr"/>
@@ -5077,7 +5077,7 @@
       </c>
       <c r="K80" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L80" s="2" t="inlineStr"/>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="K81" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L81" s="2" t="inlineStr"/>
@@ -5189,7 +5189,7 @@
       </c>
       <c r="K82" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L82" s="2" t="inlineStr"/>
@@ -5349,7 +5349,7 @@
       </c>
       <c r="K85" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L85" s="2" t="inlineStr"/>
@@ -5457,7 +5457,7 @@
       </c>
       <c r="K87" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L87" s="2" t="inlineStr"/>
@@ -5513,7 +5513,7 @@
       </c>
       <c r="K88" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L88" s="2" t="inlineStr"/>
@@ -5569,7 +5569,7 @@
       </c>
       <c r="K89" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L89" s="2" t="inlineStr"/>
@@ -5625,7 +5625,7 @@
       </c>
       <c r="K90" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L90" s="2" t="inlineStr"/>
@@ -5733,7 +5733,7 @@
       </c>
       <c r="K92" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L92" s="2" t="inlineStr"/>
@@ -5789,7 +5789,7 @@
       </c>
       <c r="K93" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L93" s="2" t="inlineStr"/>
@@ -5845,7 +5845,7 @@
       </c>
       <c r="K94" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L94" s="2" t="inlineStr"/>
@@ -5901,7 +5901,7 @@
       </c>
       <c r="K95" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L95" s="2" t="inlineStr"/>
@@ -5957,7 +5957,7 @@
       </c>
       <c r="K96" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L96" s="2" t="inlineStr"/>
@@ -6013,7 +6013,7 @@
       </c>
       <c r="K97" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L97" s="2" t="inlineStr"/>
@@ -6069,7 +6069,7 @@
       </c>
       <c r="K98" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L98" s="2" t="inlineStr"/>
@@ -6125,7 +6125,7 @@
       </c>
       <c r="K99" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L99" s="2" t="inlineStr"/>
@@ -6233,7 +6233,7 @@
       </c>
       <c r="K101" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L101" s="2" t="inlineStr"/>
@@ -6289,7 +6289,7 @@
       </c>
       <c r="K102" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L102" s="2" t="inlineStr"/>
@@ -6345,7 +6345,7 @@
       </c>
       <c r="K103" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L103" s="2" t="inlineStr"/>
@@ -6401,7 +6401,7 @@
       </c>
       <c r="K104" s="2" t="inlineStr">
         <is>
-          <t>(udfyldes — Fase C)</t>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
         </is>
       </c>
       <c r="L104" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Docs: ajourfoer godkendelsespakke + sporbarhedsmatrix (central auth, SAF-T-input, analyse-moduler, robust scope; 103 kontroller / v1.1.0)
</commit_message>
<xml_diff>
--- a/docs/VAT-Analytics_Regel-sporbarhedsmatrix.xlsx
+++ b/docs/VAT-Analytics_Regel-sporbarhedsmatrix.xlsx
@@ -1,20 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Oversigt" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sporbarhedsmatrix" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Kategorier" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oversigt" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sporbarhedsmatrix" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analyse-moduler" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kategorier" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Oversigt'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sporbarhedsmatrix'!$A$1:$L$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Kategorier'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sporbarhedsmatrix'!$A$1:$N$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Analyse-moduler'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Kategorier'!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -467,7 +469,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>1.0.0</t>
+          <t>1.1.0</t>
         </is>
       </c>
     </row>
@@ -479,7 +481,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-09-08</t>
         </is>
       </c>
     </row>
@@ -571,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L104"/>
+  <dimension ref="A1:N104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -581,11 +583,13 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="10" max="10"/>
     <col width="40" customWidth="1" min="11" max="11"/>
-    <col width="38" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="38" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -626,25 +630,35 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Analyse-modul</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Default</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Retsområde / kilde</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Modul</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Kilde-modul</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Funktion</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Dækkende test</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Afhænger af</t>
         </is>
@@ -686,25 +700,35 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
           <t>Momsgrundlag og fradragsret (momsloven) — datakvalitet jf. Skattestyrelsens kontrolmetoder</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat01_transaction_integrity.py</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>test_01_vat_recalculation</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -742,25 +766,35 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
           <t>Momsgrundlag og fradragsret (momsloven) — datakvalitet jf. Skattestyrelsens kontrolmetoder</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat01_transaction_integrity.py</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>test_02_tax_code_validation</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -798,25 +832,35 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
           <t>Momsgrundlag og fradragsret (momsloven) — datakvalitet jf. Skattestyrelsens kontrolmetoder</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat01_transaction_integrity.py</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>test_03_vat_rounding</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -854,25 +898,35 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
           <t>Momsgrundlag og fradragsret (momsloven) — datakvalitet jf. Skattestyrelsens kontrolmetoder</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat01_transaction_integrity.py</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>test_04_invoice_field_completeness</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -910,25 +964,35 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
           <t>Momsgrundlag og fradragsret (momsloven) — datakvalitet jf. Skattestyrelsens kontrolmetoder</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat01_transaction_integrity.py</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>test_05_date_consistency</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -966,25 +1030,35 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
           <t>Momsgrundlag og fradragsret (momsloven) — datakvalitet jf. Skattestyrelsens kontrolmetoder</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat01_transaction_integrity.py</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>test_06_negative_amounts</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1022,25 +1096,35 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
           <t>Momsgrundlag og fradragsret (momsloven) — datakvalitet jf. Skattestyrelsens kontrolmetoder</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat01_transaction_integrity.py</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>test_07_zero_value_transactions</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1078,25 +1162,35 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
           <t>Momsgrundlag og fradragsret (momsloven) — datakvalitet jf. Skattestyrelsens kontrolmetoder</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat01_transaction_integrity.py</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>test_08_currency_consistency</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1134,25 +1228,35 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
           <t>Momsgrundlag og fradragsret (momsloven) — datakvalitet jf. Skattestyrelsens kontrolmetoder</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat01_transaction_integrity.py</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>test_09_tax_point</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1190,25 +1294,35 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
           <t>Momsgrundlag og fradragsret (momsloven) — datakvalitet jf. Skattestyrelsens kontrolmetoder</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat01_transaction_integrity.py</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>test_10_document_type</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1246,25 +1360,35 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
           <t>Dobbelt fradrag / dublethåndtering (momsloven, fradragsret)</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat02_duplicate_detection.py</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>test_11_exact_duplicate</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1302,25 +1426,35 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
           <t>Dobbelt fradrag / dublethåndtering (momsloven, fradragsret)</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat02_duplicate_detection.py</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>test_12_fuzzy_duplicate</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1358,25 +1492,35 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
+          <t>Dublet-recovery (bredt)</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
           <t>Dobbelt fradrag / dublethåndtering (momsloven, fradragsret)</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat02_duplicate_detection.py</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>test_13_same_amount_same_vendor</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1414,25 +1558,35 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
           <t>Dobbelt fradrag / dublethåndtering (momsloven, fradragsret)</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat02_duplicate_detection.py</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>test_14_normalized_invoice_number</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1470,25 +1624,35 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
+          <t>Dublet-recovery (bredt)</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
           <t>Dobbelt fradrag / dublethåndtering (momsloven, fradragsret)</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat02_duplicate_detection.py</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>test_15_duplicate_payment</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1526,25 +1690,35 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
           <t>Dobbelt fradrag / dublethåndtering (momsloven, fradragsret)</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat02_duplicate_detection.py</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>test_16_credit_note_duplicate</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1582,25 +1756,35 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
           <t>Dobbelt fradrag / dublethåndtering (momsloven, fradragsret)</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat02_duplicate_detection.py</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>test_17_cross_entity_duplicate</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1638,25 +1822,35 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
+          <t>Dublet-recovery (bredt)</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
           <t>Dobbelt fradrag / dublethåndtering (momsloven, fradragsret)</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat02_duplicate_detection.py</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>test_18_sequential_gaps</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1694,25 +1888,35 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
           <t>Momssatser: standardsats 25% og 0-sats (momsloven)</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat03_vat_rate_validation.py</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>test_19_invalid_rate</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1750,25 +1954,35 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
           <t>Momssatser: standardsats 25% og 0-sats (momsloven)</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="K21" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat03_vat_rate_validation.py</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="L21" s="2" t="inlineStr">
         <is>
           <t>test_20_rate_vs_taxtable</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1806,25 +2020,35 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
           <t>Momssatser: standardsats 25% og 0-sats (momsloven)</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr">
+      <c r="K22" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat03_vat_rate_validation.py</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="L22" s="2" t="inlineStr">
         <is>
           <t>test_21_reduced_rate</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1862,25 +2086,35 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
           <t>Momssatser: standardsats 25% og 0-sats (momsloven)</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr">
+      <c r="K23" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat03_vat_rate_validation.py</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="L23" s="2" t="inlineStr">
         <is>
           <t>test_22_missing_output_vat</t>
         </is>
       </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1918,25 +2152,35 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
           <t>Momssatser: standardsats 25% og 0-sats (momsloven)</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="K24" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat03_vat_rate_validation.py</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
+      <c r="L24" s="2" t="inlineStr">
         <is>
           <t>test_23_rate_consistency_per_code</t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1974,25 +2218,35 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
           <t>Momssatser: standardsats 25% og 0-sats (momsloven)</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="K25" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat03_vat_rate_validation.py</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr">
+      <c r="L25" s="2" t="inlineStr">
         <is>
           <t>test_24_implied_rate</t>
         </is>
       </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2030,25 +2284,35 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
           <t>Momssatser: standardsats 25% og 0-sats (momsloven)</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat03_vat_rate_validation.py</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="L26" s="2" t="inlineStr">
         <is>
           <t>test_25_zero_rate_domestic</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2086,25 +2350,35 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
           <t>Momssatser: standardsats 25% og 0-sats (momsloven)</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="K27" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat03_vat_rate_validation.py</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
+      <c r="L27" s="2" t="inlineStr">
         <is>
           <t>test_26_missing_tax_code</t>
         </is>
       </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2142,25 +2416,35 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
           <t>Leveringssted, EU-handel og eksport: 0-sats og omvendt betalingspligt (momsloven)</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
+      <c r="K28" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat04_cross_border_eu.py</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="L28" s="2" t="inlineStr">
         <is>
           <t>test_27_eu_trade_no_vat_number</t>
         </is>
       </c>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2198,25 +2482,35 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
           <t>Leveringssted, EU-handel og eksport: 0-sats og omvendt betalingspligt (momsloven)</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
+      <c r="K29" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat04_cross_border_eu.py</t>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr">
+      <c r="L29" s="2" t="inlineStr">
         <is>
           <t>test_28_invalid_eu_vat_format</t>
         </is>
       </c>
-      <c r="K29" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2254,25 +2548,35 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
           <t>Leveringssted, EU-handel og eksport: 0-sats og omvendt betalingspligt (momsloven)</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr">
+      <c r="K30" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat04_cross_border_eu.py</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr">
+      <c r="L30" s="2" t="inlineStr">
         <is>
           <t>test_29_eu_acquisition_no_reverse_charge</t>
         </is>
       </c>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2310,25 +2614,35 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
           <t>Leveringssted, EU-handel og eksport: 0-sats og omvendt betalingspligt (momsloven)</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr">
+      <c r="K31" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat04_cross_border_eu.py</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr">
+      <c r="L31" s="2" t="inlineStr">
         <is>
           <t>test_30_export_with_vat</t>
         </is>
       </c>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L31" s="2" t="inlineStr"/>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2366,25 +2680,35 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
           <t>Leveringssted, EU-handel og eksport: 0-sats og omvendt betalingspligt (momsloven)</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr">
+      <c r="K32" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat04_cross_border_eu.py</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr">
+      <c r="L32" s="2" t="inlineStr">
         <is>
           <t>test_31_eu_sale_with_dk_vat</t>
         </is>
       </c>
-      <c r="K32" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L32" s="2" t="inlineStr"/>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2422,25 +2746,35 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
           <t>Leveringssted, EU-handel og eksport: 0-sats og omvendt betalingspligt (momsloven)</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr">
+      <c r="K33" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat04_cross_border_eu.py</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr">
+      <c r="L33" s="2" t="inlineStr">
         <is>
           <t>test_32_missing_country_on_foreign</t>
         </is>
       </c>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2478,25 +2812,35 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
           <t>Leveringssted, EU-handel og eksport: 0-sats og omvendt betalingspligt (momsloven)</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr">
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat04_cross_border_eu.py</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr">
+      <c r="L34" s="2" t="inlineStr">
         <is>
           <t>test_33_currency_country_mismatch</t>
         </is>
       </c>
-      <c r="K34" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L34" s="2" t="inlineStr"/>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2534,25 +2878,35 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
           <t>Leveringssted, EU-handel og eksport: 0-sats og omvendt betalingspligt (momsloven)</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr">
+      <c r="K35" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat04_cross_border_eu.py</t>
         </is>
       </c>
-      <c r="J35" s="2" t="inlineStr">
+      <c r="L35" s="2" t="inlineStr">
         <is>
           <t>test_34_dk_vat_on_foreign_party</t>
         </is>
       </c>
-      <c r="K35" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L35" s="2" t="inlineStr"/>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2590,25 +2944,35 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
           <t>Leveringssted, EU-handel og eksport: 0-sats og omvendt betalingspligt (momsloven)</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr">
+      <c r="K36" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat04_cross_border_eu.py</t>
         </is>
       </c>
-      <c r="J36" s="2" t="inlineStr">
+      <c r="L36" s="2" t="inlineStr">
         <is>
           <t>test_35_vat_prefix_vs_country</t>
         </is>
       </c>
-      <c r="K36" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L36" s="2" t="inlineStr"/>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2646,25 +3010,35 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
           <t>Leveringssted, EU-handel og eksport: 0-sats og omvendt betalingspligt (momsloven)</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr">
+      <c r="K37" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat04_cross_border_eu.py</t>
         </is>
       </c>
-      <c r="J37" s="2" t="inlineStr">
+      <c r="L37" s="2" t="inlineStr">
         <is>
           <t>test_36_triangulation</t>
         </is>
       </c>
-      <c r="K37" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L37" s="2" t="inlineStr">
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr">
         <is>
           <t>ship_from_country / ship_to_country (vareflow)</t>
         </is>
@@ -2706,25 +3080,35 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
           <t>Leveringssted, EU-handel og eksport: 0-sats og omvendt betalingspligt (momsloven)</t>
         </is>
       </c>
-      <c r="I38" s="2" t="inlineStr">
+      <c r="K38" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat04_cross_border_eu.py</t>
         </is>
       </c>
-      <c r="J38" s="2" t="inlineStr">
+      <c r="L38" s="2" t="inlineStr">
         <is>
           <t>test_37_vies_verification</t>
         </is>
       </c>
-      <c r="K38" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L38" s="2" t="inlineStr"/>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2762,25 +3146,35 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
           <t>Leveringssted, EU-handel og eksport: 0-sats og omvendt betalingspligt (momsloven)</t>
         </is>
       </c>
-      <c r="I39" s="2" t="inlineStr">
+      <c r="K39" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat04_cross_border_eu.py</t>
         </is>
       </c>
-      <c r="J39" s="2" t="inlineStr">
+      <c r="L39" s="2" t="inlineStr">
         <is>
           <t>test_38_import_without_docs</t>
         </is>
       </c>
-      <c r="K39" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L39" s="2" t="inlineStr"/>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2818,25 +3212,35 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
           <t>Leveringstidspunkt og angivelsesperiode — periodisering (momsloven)</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr">
+      <c r="K40" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat05_timing_period.py</t>
         </is>
       </c>
-      <c r="J40" s="2" t="inlineStr">
+      <c r="L40" s="2" t="inlineStr">
         <is>
           <t>test_39_after_period_end</t>
         </is>
       </c>
-      <c r="K40" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L40" s="2" t="inlineStr"/>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2874,25 +3278,35 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
           <t>Leveringstidspunkt og angivelsesperiode — periodisering (momsloven)</t>
         </is>
       </c>
-      <c r="I41" s="2" t="inlineStr">
+      <c r="K41" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat05_timing_period.py</t>
         </is>
       </c>
-      <c r="J41" s="2" t="inlineStr">
+      <c r="L41" s="2" t="inlineStr">
         <is>
           <t>test_40_before_period_start</t>
         </is>
       </c>
-      <c r="K41" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L41" s="2" t="inlineStr"/>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2930,25 +3344,35 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
           <t>Leveringstidspunkt og angivelsesperiode — periodisering (momsloven)</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr">
+      <c r="K42" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat05_timing_period.py</t>
         </is>
       </c>
-      <c r="J42" s="2" t="inlineStr">
+      <c r="L42" s="2" t="inlineStr">
         <is>
           <t>test_41_weekend_postings</t>
         </is>
       </c>
-      <c r="K42" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L42" s="2" t="inlineStr"/>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2986,25 +3410,35 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
           <t>Leveringstidspunkt og angivelsesperiode — periodisering (momsloven)</t>
         </is>
       </c>
-      <c r="I43" s="2" t="inlineStr">
+      <c r="K43" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat05_timing_period.py</t>
         </is>
       </c>
-      <c r="J43" s="2" t="inlineStr">
+      <c r="L43" s="2" t="inlineStr">
         <is>
           <t>test_42_period_end_clustering</t>
         </is>
       </c>
-      <c r="K43" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L43" s="2" t="inlineStr"/>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3042,25 +3476,35 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
           <t>Leveringstidspunkt og angivelsesperiode — periodisering (momsloven)</t>
         </is>
       </c>
-      <c r="I44" s="2" t="inlineStr">
+      <c r="K44" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat05_timing_period.py</t>
         </is>
       </c>
-      <c r="J44" s="2" t="inlineStr">
+      <c r="L44" s="2" t="inlineStr">
         <is>
           <t>test_43_future_dates</t>
         </is>
       </c>
-      <c r="K44" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L44" s="2" t="inlineStr"/>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3098,25 +3542,35 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
           <t>Leveringstidspunkt og angivelsesperiode — periodisering (momsloven)</t>
         </is>
       </c>
-      <c r="I45" s="2" t="inlineStr">
+      <c r="K45" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat05_timing_period.py</t>
         </is>
       </c>
-      <c r="J45" s="2" t="inlineStr">
+      <c r="L45" s="2" t="inlineStr">
         <is>
           <t>test_44_period_boundary</t>
         </is>
       </c>
-      <c r="K45" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L45" s="2" t="inlineStr"/>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3154,25 +3608,35 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
           <t>Leveringstidspunkt og angivelsesperiode — periodisering (momsloven)</t>
         </is>
       </c>
-      <c r="I46" s="2" t="inlineStr">
+      <c r="K46" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat05_timing_period.py</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr">
+      <c r="L46" s="2" t="inlineStr">
         <is>
           <t>test_45_sequence_vs_date</t>
         </is>
       </c>
-      <c r="K46" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L46" s="2" t="inlineStr"/>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3210,25 +3674,35 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
           <t>Leveringstidspunkt og angivelsesperiode — periodisering (momsloven)</t>
         </is>
       </c>
-      <c r="I47" s="2" t="inlineStr">
+      <c r="K47" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat05_timing_period.py</t>
         </is>
       </c>
-      <c r="J47" s="2" t="inlineStr">
+      <c r="L47" s="2" t="inlineStr">
         <is>
           <t>test_46_invoice_posting_lag</t>
         </is>
       </c>
-      <c r="K47" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L47" s="2" t="inlineStr">
+      <c r="M47" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N47" s="2" t="inlineStr">
         <is>
           <t>to datoer: bogføringsdato + fakturadato</t>
         </is>
@@ -3270,25 +3744,35 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
+          <t>Stamdata- &amp; datakvalitet</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
           <t>Gyldigt momsnummer og parts-/fakturakrav (momsloven, VIES)</t>
         </is>
       </c>
-      <c r="I48" s="2" t="inlineStr">
+      <c r="K48" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat06_party_validation.py</t>
         </is>
       </c>
-      <c r="J48" s="2" t="inlineStr">
+      <c r="L48" s="2" t="inlineStr">
         <is>
           <t>test_47_missing_party_name</t>
         </is>
       </c>
-      <c r="K48" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L48" s="2" t="inlineStr"/>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3326,25 +3810,35 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
+          <t>Stamdata- &amp; datakvalitet</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
           <t>Gyldigt momsnummer og parts-/fakturakrav (momsloven, VIES)</t>
         </is>
       </c>
-      <c r="I49" s="2" t="inlineStr">
+      <c r="K49" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat06_party_validation.py</t>
         </is>
       </c>
-      <c r="J49" s="2" t="inlineStr">
+      <c r="L49" s="2" t="inlineStr">
         <is>
           <t>test_48_duplicate_suppliers</t>
         </is>
       </c>
-      <c r="K49" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L49" s="2" t="inlineStr"/>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3382,25 +3876,35 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
           <t>Gyldigt momsnummer og parts-/fakturakrav (momsloven, VIES)</t>
         </is>
       </c>
-      <c r="I50" s="2" t="inlineStr">
+      <c r="K50" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat06_party_validation.py</t>
         </is>
       </c>
-      <c r="J50" s="2" t="inlineStr">
+      <c r="L50" s="2" t="inlineStr">
         <is>
           <t>test_49_missing_cvr_dk_supplier</t>
         </is>
       </c>
-      <c r="K50" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L50" s="2" t="inlineStr"/>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3438,25 +3942,35 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
           <t>Gyldigt momsnummer og parts-/fakturakrav (momsloven, VIES)</t>
         </is>
       </c>
-      <c r="I51" s="2" t="inlineStr">
+      <c r="K51" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat06_party_validation.py</t>
         </is>
       </c>
-      <c r="J51" s="2" t="inlineStr">
+      <c r="L51" s="2" t="inlineStr">
         <is>
           <t>test_50_invalid_cvr_format</t>
         </is>
       </c>
-      <c r="K51" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L51" s="2" t="inlineStr"/>
+      <c r="M51" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3494,25 +4008,35 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
+          <t>Stamdata- &amp; datakvalitet</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
           <t>Gyldigt momsnummer og parts-/fakturakrav (momsloven, VIES)</t>
         </is>
       </c>
-      <c r="I52" s="2" t="inlineStr">
+      <c r="K52" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat06_party_validation.py</t>
         </is>
       </c>
-      <c r="J52" s="2" t="inlineStr">
+      <c r="L52" s="2" t="inlineStr">
         <is>
           <t>test_51_one_off_supplier</t>
         </is>
       </c>
-      <c r="K52" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L52" s="2" t="inlineStr"/>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3550,25 +4074,35 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
           <t>Gyldigt momsnummer og parts-/fakturakrav (momsloven, VIES)</t>
         </is>
       </c>
-      <c r="I53" s="2" t="inlineStr">
+      <c r="K53" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat06_party_validation.py</t>
         </is>
       </c>
-      <c r="J53" s="2" t="inlineStr">
+      <c r="L53" s="2" t="inlineStr">
         <is>
           <t>test_52_customer_without_vat</t>
         </is>
       </c>
-      <c r="K53" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L53" s="2" t="inlineStr"/>
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3606,25 +4140,35 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
           <t>Gyldigt momsnummer og parts-/fakturakrav (momsloven, VIES)</t>
         </is>
       </c>
-      <c r="I54" s="2" t="inlineStr">
+      <c r="K54" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat06_party_validation.py</t>
         </is>
       </c>
-      <c r="J54" s="2" t="inlineStr">
+      <c r="L54" s="2" t="inlineStr">
         <is>
           <t>test_53_shared_identity</t>
         </is>
       </c>
-      <c r="K54" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L54" s="2" t="inlineStr"/>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3662,25 +4206,35 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
+          <t>Stamdata- &amp; datakvalitet</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
           <t>Gyldigt momsnummer og parts-/fakturakrav (momsloven, VIES)</t>
         </is>
       </c>
-      <c r="I55" s="2" t="inlineStr">
+      <c r="K55" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat06_party_validation.py</t>
         </is>
       </c>
-      <c r="J55" s="2" t="inlineStr">
+      <c r="L55" s="2" t="inlineStr">
         <is>
           <t>test_54_party_in_both_roles</t>
         </is>
       </c>
-      <c r="K55" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L55" s="2" t="inlineStr"/>
+      <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3718,25 +4272,35 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
           <t>Beløbs- og tærskelkontroller (Skattestyrelsens kontrolmetoder)</t>
         </is>
       </c>
-      <c r="I56" s="2" t="inlineStr">
+      <c r="K56" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat07_amount_threshold.py</t>
         </is>
       </c>
-      <c r="J56" s="2" t="inlineStr">
+      <c r="L56" s="2" t="inlineStr">
         <is>
           <t>test_55_round_amounts</t>
         </is>
       </c>
-      <c r="K56" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L56" s="2" t="inlineStr"/>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3774,25 +4338,35 @@
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
           <t>Beløbs- og tærskelkontroller (Skattestyrelsens kontrolmetoder)</t>
         </is>
       </c>
-      <c r="I57" s="2" t="inlineStr">
+      <c r="K57" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat07_amount_threshold.py</t>
         </is>
       </c>
-      <c r="J57" s="2" t="inlineStr">
+      <c r="L57" s="2" t="inlineStr">
         <is>
           <t>test_56_just_below_threshold</t>
         </is>
       </c>
-      <c r="K57" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L57" s="2" t="inlineStr"/>
+      <c r="M57" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3830,25 +4404,35 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
           <t>Beløbs- og tærskelkontroller (Skattestyrelsens kontrolmetoder)</t>
         </is>
       </c>
-      <c r="I58" s="2" t="inlineStr">
+      <c r="K58" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat07_amount_threshold.py</t>
         </is>
       </c>
-      <c r="J58" s="2" t="inlineStr">
+      <c r="L58" s="2" t="inlineStr">
         <is>
           <t>test_57_cash_limit</t>
         </is>
       </c>
-      <c r="K58" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L58" s="2" t="inlineStr"/>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -3886,25 +4470,35 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
           <t>Beløbs- og tærskelkontroller (Skattestyrelsens kontrolmetoder)</t>
         </is>
       </c>
-      <c r="I59" s="2" t="inlineStr">
+      <c r="K59" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat07_amount_threshold.py</t>
         </is>
       </c>
-      <c r="J59" s="2" t="inlineStr">
+      <c r="L59" s="2" t="inlineStr">
         <is>
           <t>test_58_unusually_large</t>
         </is>
       </c>
-      <c r="K59" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L59" s="2" t="inlineStr"/>
+      <c r="M59" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3942,25 +4536,35 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
           <t>Beløbs- og tærskelkontroller (Skattestyrelsens kontrolmetoder)</t>
         </is>
       </c>
-      <c r="I60" s="2" t="inlineStr">
+      <c r="K60" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat07_amount_threshold.py</t>
         </is>
       </c>
-      <c r="J60" s="2" t="inlineStr">
+      <c r="L60" s="2" t="inlineStr">
         <is>
           <t>test_59_large_vat_no_document</t>
         </is>
       </c>
-      <c r="K60" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L60" s="2" t="inlineStr"/>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -3998,25 +4602,35 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
           <t>Beløbs- og tærskelkontroller (Skattestyrelsens kontrolmetoder)</t>
         </is>
       </c>
-      <c r="I61" s="2" t="inlineStr">
+      <c r="K61" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat07_amount_threshold.py</t>
         </is>
       </c>
-      <c r="J61" s="2" t="inlineStr">
+      <c r="L61" s="2" t="inlineStr">
         <is>
           <t>test_60_negative_vat</t>
         </is>
       </c>
-      <c r="K61" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L61" s="2" t="inlineStr"/>
+      <c r="M61" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -4054,25 +4668,35 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
           <t>Beløbs- og tærskelkontroller (Skattestyrelsens kontrolmetoder)</t>
         </is>
       </c>
-      <c r="I62" s="2" t="inlineStr">
+      <c r="K62" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat07_amount_threshold.py</t>
         </is>
       </c>
-      <c r="J62" s="2" t="inlineStr">
+      <c r="L62" s="2" t="inlineStr">
         <is>
           <t>test_61_account_outlier</t>
         </is>
       </c>
-      <c r="K62" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L62" s="2" t="inlineStr"/>
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -4110,25 +4734,35 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
           <t>Beløbs- og tærskelkontroller (Skattestyrelsens kontrolmetoder)</t>
         </is>
       </c>
-      <c r="I63" s="2" t="inlineStr">
+      <c r="K63" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat07_amount_threshold.py</t>
         </is>
       </c>
-      <c r="J63" s="2" t="inlineStr">
+      <c r="L63" s="2" t="inlineStr">
         <is>
           <t>test_62_structuring</t>
         </is>
       </c>
-      <c r="K63" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L63" s="2" t="inlineStr"/>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -4166,25 +4800,35 @@
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
           <t>Statistisk anomalidetektion, Benford m.v. (Skattestyrelsens kontrolmetoder)</t>
         </is>
       </c>
-      <c r="I64" s="2" t="inlineStr">
+      <c r="K64" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat08_statistical_anomaly.py</t>
         </is>
       </c>
-      <c r="J64" s="2" t="inlineStr">
+      <c r="L64" s="2" t="inlineStr">
         <is>
           <t>test_63_benford_first_digit</t>
         </is>
       </c>
-      <c r="K64" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L64" s="2" t="inlineStr"/>
+      <c r="M64" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -4222,25 +4866,35 @@
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
           <t>Statistisk anomalidetektion, Benford m.v. (Skattestyrelsens kontrolmetoder)</t>
         </is>
       </c>
-      <c r="I65" s="2" t="inlineStr">
+      <c r="K65" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat08_statistical_anomaly.py</t>
         </is>
       </c>
-      <c r="J65" s="2" t="inlineStr">
+      <c r="L65" s="2" t="inlineStr">
         <is>
           <t>test_64_round_number_bias</t>
         </is>
       </c>
-      <c r="K65" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L65" s="2" t="inlineStr"/>
+      <c r="M65" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -4278,25 +4932,35 @@
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
           <t>Statistisk anomalidetektion, Benford m.v. (Skattestyrelsens kontrolmetoder)</t>
         </is>
       </c>
-      <c r="I66" s="2" t="inlineStr">
+      <c r="K66" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat08_statistical_anomaly.py</t>
         </is>
       </c>
-      <c r="J66" s="2" t="inlineStr">
+      <c r="L66" s="2" t="inlineStr">
         <is>
           <t>test_65_rare_tax_code</t>
         </is>
       </c>
-      <c r="K66" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L66" s="2" t="inlineStr"/>
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -4334,25 +4998,35 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
           <t>Statistisk anomalidetektion, Benford m.v. (Skattestyrelsens kontrolmetoder)</t>
         </is>
       </c>
-      <c r="I67" s="2" t="inlineStr">
+      <c r="K67" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat08_statistical_anomaly.py</t>
         </is>
       </c>
-      <c r="J67" s="2" t="inlineStr">
+      <c r="L67" s="2" t="inlineStr">
         <is>
           <t>test_66_duplicate_descriptions</t>
         </is>
       </c>
-      <c r="K67" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L67" s="2" t="inlineStr"/>
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N67" s="2" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -4390,25 +5064,35 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
           <t>Statistisk anomalidetektion, Benford m.v. (Skattestyrelsens kontrolmetoder)</t>
         </is>
       </c>
-      <c r="I68" s="2" t="inlineStr">
+      <c r="K68" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat08_statistical_anomaly.py</t>
         </is>
       </c>
-      <c r="J68" s="2" t="inlineStr">
+      <c r="L68" s="2" t="inlineStr">
         <is>
           <t>test_67_timeseries_spike</t>
         </is>
       </c>
-      <c r="K68" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L68" s="2" t="inlineStr"/>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -4446,25 +5130,35 @@
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
           <t>Statistisk anomalidetektion, Benford m.v. (Skattestyrelsens kontrolmetoder)</t>
         </is>
       </c>
-      <c r="I69" s="2" t="inlineStr">
+      <c r="K69" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat08_statistical_anomaly.py</t>
         </is>
       </c>
-      <c r="J69" s="2" t="inlineStr">
+      <c r="L69" s="2" t="inlineStr">
         <is>
           <t>test_68_rare_account</t>
         </is>
       </c>
-      <c r="K69" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L69" s="2" t="inlineStr"/>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N69" s="2" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -4502,25 +5196,35 @@
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
           <t>Statistisk anomalidetektion, Benford m.v. (Skattestyrelsens kontrolmetoder)</t>
         </is>
       </c>
-      <c r="I70" s="2" t="inlineStr">
+      <c r="K70" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat08_statistical_anomaly.py</t>
         </is>
       </c>
-      <c r="J70" s="2" t="inlineStr">
+      <c r="L70" s="2" t="inlineStr">
         <is>
           <t>test_69_last_digit_uniformity</t>
         </is>
       </c>
-      <c r="K70" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L70" s="2" t="inlineStr"/>
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N70" s="2" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -4558,25 +5262,35 @@
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
           <t>Omvendt betalingspligt / reverse charge (momsloven)</t>
         </is>
       </c>
-      <c r="I71" s="2" t="inlineStr">
+      <c r="K71" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat09_reverse_charge.py</t>
         </is>
       </c>
-      <c r="J71" s="2" t="inlineStr">
+      <c r="L71" s="2" t="inlineStr">
         <is>
           <t>test_70_eu_service_no_rc</t>
         </is>
       </c>
-      <c r="K71" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L71" s="2" t="inlineStr"/>
+      <c r="M71" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4614,25 +5328,35 @@
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
           <t>Omvendt betalingspligt / reverse charge (momsloven)</t>
         </is>
       </c>
-      <c r="I72" s="2" t="inlineStr">
+      <c r="K72" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat09_reverse_charge.py</t>
         </is>
       </c>
-      <c r="J72" s="2" t="inlineStr">
+      <c r="L72" s="2" t="inlineStr">
         <is>
           <t>test_71_rc_on_domestic</t>
         </is>
       </c>
-      <c r="K72" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L72" s="2" t="inlineStr"/>
+      <c r="M72" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -4670,25 +5394,35 @@
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
           <t>Omvendt betalingspligt / reverse charge (momsloven)</t>
         </is>
       </c>
-      <c r="I73" s="2" t="inlineStr">
+      <c r="K73" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat09_reverse_charge.py</t>
         </is>
       </c>
-      <c r="J73" s="2" t="inlineStr">
+      <c r="L73" s="2" t="inlineStr">
         <is>
           <t>test_72_domestic_rc_goods</t>
         </is>
       </c>
-      <c r="K73" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L73" s="2" t="inlineStr"/>
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -4726,25 +5460,35 @@
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
           <t>Omvendt betalingspligt / reverse charge (momsloven)</t>
         </is>
       </c>
-      <c r="I74" s="2" t="inlineStr">
+      <c r="K74" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat09_reverse_charge.py</t>
         </is>
       </c>
-      <c r="J74" s="2" t="inlineStr">
+      <c r="L74" s="2" t="inlineStr">
         <is>
           <t>test_73_asymmetric_rc</t>
         </is>
       </c>
-      <c r="K74" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L74" s="2" t="inlineStr"/>
+      <c r="M74" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N74" s="2" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -4782,25 +5526,35 @@
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
           <t>Omvendt betalingspligt / reverse charge (momsloven)</t>
         </is>
       </c>
-      <c r="I75" s="2" t="inlineStr">
+      <c r="K75" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat09_reverse_charge.py</t>
         </is>
       </c>
-      <c r="J75" s="2" t="inlineStr">
+      <c r="L75" s="2" t="inlineStr">
         <is>
           <t>test_74_construction_rc</t>
         </is>
       </c>
-      <c r="K75" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L75" s="2" t="inlineStr"/>
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N75" s="2" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -4838,25 +5592,35 @@
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
           <t>Omvendt betalingspligt / reverse charge (momsloven)</t>
         </is>
       </c>
-      <c r="I76" s="2" t="inlineStr">
+      <c r="K76" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat09_reverse_charge.py</t>
         </is>
       </c>
-      <c r="J76" s="2" t="inlineStr">
+      <c r="L76" s="2" t="inlineStr">
         <is>
           <t>test_75_rc_missing_documentation</t>
         </is>
       </c>
-      <c r="K76" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L76" s="2" t="inlineStr"/>
+      <c r="M76" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N76" s="2" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -4894,25 +5658,35 @@
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
           <t>Opgørelse og afstemning af ind-/udgående moms; (delvis) fradragsret (momsloven)</t>
         </is>
       </c>
-      <c r="I77" s="2" t="inlineStr">
+      <c r="K77" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat10_vat_reconciliation.py</t>
         </is>
       </c>
-      <c r="J77" s="2" t="inlineStr">
+      <c r="L77" s="2" t="inlineStr">
         <is>
           <t>test_76_input_output_ratio</t>
         </is>
       </c>
-      <c r="K77" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L77" s="2" t="inlineStr"/>
+      <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -4950,25 +5724,35 @@
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
           <t>Opgørelse og afstemning af ind-/udgående moms; (delvis) fradragsret (momsloven)</t>
         </is>
       </c>
-      <c r="I78" s="2" t="inlineStr">
+      <c r="K78" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat10_vat_reconciliation.py</t>
         </is>
       </c>
-      <c r="J78" s="2" t="inlineStr">
+      <c r="L78" s="2" t="inlineStr">
         <is>
           <t>test_77_vat_account_reconciliation</t>
         </is>
       </c>
-      <c r="K78" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L78" s="2" t="inlineStr"/>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N78" s="2" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -5006,25 +5790,35 @@
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
           <t>Opgørelse og afstemning af ind-/udgående moms; (delvis) fradragsret (momsloven)</t>
         </is>
       </c>
-      <c r="I79" s="2" t="inlineStr">
+      <c r="K79" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat10_vat_reconciliation.py</t>
         </is>
       </c>
-      <c r="J79" s="2" t="inlineStr">
+      <c r="L79" s="2" t="inlineStr">
         <is>
           <t>test_78_negative_vat_liability</t>
         </is>
       </c>
-      <c r="K79" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L79" s="2" t="inlineStr"/>
+      <c r="M79" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N79" s="2" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -5062,25 +5856,35 @@
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
           <t>Opgørelse og afstemning af ind-/udgående moms; (delvis) fradragsret (momsloven)</t>
         </is>
       </c>
-      <c r="I80" s="2" t="inlineStr">
+      <c r="K80" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat10_vat_reconciliation.py</t>
         </is>
       </c>
-      <c r="J80" s="2" t="inlineStr">
+      <c r="L80" s="2" t="inlineStr">
         <is>
           <t>test_79_input_vat_no_purchase</t>
         </is>
       </c>
-      <c r="K80" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L80" s="2" t="inlineStr"/>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N80" s="2" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -5118,25 +5922,35 @@
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
           <t>Opgørelse og afstemning af ind-/udgående moms; (delvis) fradragsret (momsloven)</t>
         </is>
       </c>
-      <c r="I81" s="2" t="inlineStr">
+      <c r="K81" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat10_vat_reconciliation.py</t>
         </is>
       </c>
-      <c r="J81" s="2" t="inlineStr">
+      <c r="L81" s="2" t="inlineStr">
         <is>
           <t>test_80_revenue_without_output_vat</t>
         </is>
       </c>
-      <c r="K81" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L81" s="2" t="inlineStr"/>
+      <c r="M81" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N81" s="2" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -5174,25 +5988,35 @@
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
           <t>Opgørelse og afstemning af ind-/udgående moms; (delvis) fradragsret (momsloven)</t>
         </is>
       </c>
-      <c r="I82" s="2" t="inlineStr">
+      <c r="K82" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat10_vat_reconciliation.py</t>
         </is>
       </c>
-      <c r="J82" s="2" t="inlineStr">
+      <c r="L82" s="2" t="inlineStr">
         <is>
           <t>test_81_zero_rated_share</t>
         </is>
       </c>
-      <c r="K82" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L82" s="2" t="inlineStr"/>
+      <c r="M82" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N82" s="2" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -5222,25 +6046,35 @@
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
           <t>Opgørelse og afstemning af ind-/udgående moms; (delvis) fradragsret (momsloven)</t>
         </is>
       </c>
-      <c r="I83" s="2" t="inlineStr">
+      <c r="K83" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat10_vat_reconciliation.py</t>
         </is>
       </c>
-      <c r="J83" s="2" t="inlineStr">
+      <c r="L83" s="2" t="inlineStr">
         <is>
           <t>test_82_period_declaration</t>
         </is>
       </c>
-      <c r="K83" s="2" t="inlineStr">
+      <c r="M83" s="2" t="inlineStr">
         <is>
           <t>(udfyldes — Fase C)</t>
         </is>
       </c>
-      <c r="L83" s="2" t="inlineStr">
+      <c r="N83" s="2" t="inlineStr">
         <is>
           <t>indberettet momsangivelse for perioden</t>
         </is>
@@ -5274,25 +6108,35 @@
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
           <t>Opgørelse og afstemning af ind-/udgående moms; (delvis) fradragsret (momsloven)</t>
         </is>
       </c>
-      <c r="I84" s="2" t="inlineStr">
+      <c r="K84" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat10_vat_reconciliation.py</t>
         </is>
       </c>
-      <c r="J84" s="2" t="inlineStr">
+      <c r="L84" s="2" t="inlineStr">
         <is>
           <t>test_83_partial_deduction</t>
         </is>
       </c>
-      <c r="K84" s="2" t="inlineStr">
+      <c r="M84" s="2" t="inlineStr">
         <is>
           <t>(udfyldes — Fase C)</t>
         </is>
       </c>
-      <c r="L84" s="2" t="inlineStr">
+      <c r="N84" s="2" t="inlineStr">
         <is>
           <t>delvis fradragsret (fordelingsnøgle)</t>
         </is>
@@ -5334,25 +6178,35 @@
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
           <t>Svig/MTIC: solidarisk hæftelse og karruselindikatorer (momsloven, EU)</t>
         </is>
       </c>
-      <c r="I85" s="2" t="inlineStr">
+      <c r="K85" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat11_fraud_mtic.py</t>
         </is>
       </c>
-      <c r="J85" s="2" t="inlineStr">
+      <c r="L85" s="2" t="inlineStr">
         <is>
           <t>test_84_missing_trader</t>
         </is>
       </c>
-      <c r="K85" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L85" s="2" t="inlineStr"/>
+      <c r="M85" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N85" s="2" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -5382,25 +6236,35 @@
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
           <t>Svig/MTIC: solidarisk hæftelse og karruselindikatorer (momsloven, EU)</t>
         </is>
       </c>
-      <c r="I86" s="2" t="inlineStr">
+      <c r="K86" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat11_fraud_mtic.py</t>
         </is>
       </c>
-      <c r="J86" s="2" t="inlineStr">
+      <c r="L86" s="2" t="inlineStr">
         <is>
           <t>test_85_carousel_pattern</t>
         </is>
       </c>
-      <c r="K86" s="2" t="inlineStr">
+      <c r="M86" s="2" t="inlineStr">
         <is>
           <t>(udfyldes — Fase C)</t>
         </is>
       </c>
-      <c r="L86" s="2" t="inlineStr">
+      <c r="N86" s="2" t="inlineStr">
         <is>
           <t>vareflow på tværs af virksomheder (multi-entity)</t>
         </is>
@@ -5442,25 +6306,35 @@
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
           <t>Svig/MTIC: solidarisk hæftelse og karruselindikatorer (momsloven, EU)</t>
         </is>
       </c>
-      <c r="I87" s="2" t="inlineStr">
+      <c r="K87" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat11_fraud_mtic.py</t>
         </is>
       </c>
-      <c r="J87" s="2" t="inlineStr">
+      <c r="L87" s="2" t="inlineStr">
         <is>
           <t>test_86_rapid_throughput</t>
         </is>
       </c>
-      <c r="K87" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L87" s="2" t="inlineStr"/>
+      <c r="M87" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N87" s="2" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -5498,25 +6372,35 @@
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
           <t>Svig/MTIC: solidarisk hæftelse og karruselindikatorer (momsloven, EU)</t>
         </is>
       </c>
-      <c r="I88" s="2" t="inlineStr">
+      <c r="K88" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat11_fraud_mtic.py</t>
         </is>
       </c>
-      <c r="J88" s="2" t="inlineStr">
+      <c r="L88" s="2" t="inlineStr">
         <is>
           <t>test_87_high_risk_goods</t>
         </is>
       </c>
-      <c r="K88" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L88" s="2" t="inlineStr"/>
+      <c r="M88" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N88" s="2" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -5554,25 +6438,35 @@
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
           <t>Svig/MTIC: solidarisk hæftelse og karruselindikatorer (momsloven, EU)</t>
         </is>
       </c>
-      <c r="I89" s="2" t="inlineStr">
+      <c r="K89" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat11_fraud_mtic.py</t>
         </is>
       </c>
-      <c r="J89" s="2" t="inlineStr">
+      <c r="L89" s="2" t="inlineStr">
         <is>
           <t>test_88_zero_margin</t>
         </is>
       </c>
-      <c r="K89" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L89" s="2" t="inlineStr"/>
+      <c r="M89" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N89" s="2" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -5610,25 +6504,35 @@
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
           <t>Svig/MTIC: solidarisk hæftelse og karruselindikatorer (momsloven, EU)</t>
         </is>
       </c>
-      <c r="I90" s="2" t="inlineStr">
+      <c r="K90" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat11_fraud_mtic.py</t>
         </is>
       </c>
-      <c r="J90" s="2" t="inlineStr">
+      <c r="L90" s="2" t="inlineStr">
         <is>
           <t>test_89_new_high_volume_party</t>
         </is>
       </c>
-      <c r="K90" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L90" s="2" t="inlineStr"/>
+      <c r="M90" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N90" s="2" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -5658,25 +6562,35 @@
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
           <t>Svig/MTIC: solidarisk hæftelse og karruselindikatorer (momsloven, EU)</t>
         </is>
       </c>
-      <c r="I91" s="2" t="inlineStr">
+      <c r="K91" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat11_fraud_mtic.py</t>
         </is>
       </c>
-      <c r="J91" s="2" t="inlineStr">
+      <c r="L91" s="2" t="inlineStr">
         <is>
           <t>test_90_payment_pattern</t>
         </is>
       </c>
-      <c r="K91" s="2" t="inlineStr">
+      <c r="M91" s="2" t="inlineStr">
         <is>
           <t>(udfyldes — Fase C)</t>
         </is>
       </c>
-      <c r="L91" s="2" t="inlineStr">
+      <c r="N91" s="2" t="inlineStr">
         <is>
           <t>fuld betalingsdata (modtagerkonto, betalingsdato, tredjepart)</t>
         </is>
@@ -5718,25 +6632,35 @@
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
           <t>Svig/MTIC: solidarisk hæftelse og karruselindikatorer (momsloven, EU)</t>
         </is>
       </c>
-      <c r="I92" s="2" t="inlineStr">
+      <c r="K92" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat11_fraud_mtic.py</t>
         </is>
       </c>
-      <c r="J92" s="2" t="inlineStr">
+      <c r="L92" s="2" t="inlineStr">
         <is>
           <t>test_91_clearing_account_abuse</t>
         </is>
       </c>
-      <c r="K92" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L92" s="2" t="inlineStr"/>
+      <c r="M92" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N92" s="2" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -5774,25 +6698,35 @@
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I93" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J93" s="2" t="inlineStr">
+        <is>
           <t>Svig/MTIC: solidarisk hæftelse og karruselindikatorer (momsloven, EU)</t>
         </is>
       </c>
-      <c r="I93" s="2" t="inlineStr">
+      <c r="K93" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat11_fraud_mtic.py</t>
         </is>
       </c>
-      <c r="J93" s="2" t="inlineStr">
+      <c r="L93" s="2" t="inlineStr">
         <is>
           <t>test_92_false_invoice</t>
         </is>
       </c>
-      <c r="K93" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L93" s="2" t="inlineStr"/>
+      <c r="M93" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N93" s="2" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -5830,25 +6764,35 @@
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="I94" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
           <t>Svig/MTIC: solidarisk hæftelse og karruselindikatorer (momsloven, EU)</t>
         </is>
       </c>
-      <c r="I94" s="2" t="inlineStr">
+      <c r="K94" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat11_fraud_mtic.py</t>
         </is>
       </c>
-      <c r="J94" s="2" t="inlineStr">
+      <c r="L94" s="2" t="inlineStr">
         <is>
           <t>test_93_identical_amounts_across_parties</t>
         </is>
       </c>
-      <c r="K94" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L94" s="2" t="inlineStr"/>
+      <c r="M94" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N94" s="2" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -5886,25 +6830,35 @@
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
+          <t>E-handel &amp; særordninger</t>
+        </is>
+      </c>
+      <c r="I95" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J95" s="2" t="inlineStr">
+        <is>
           <t>E-handel, digitale ydelser og særordninger: OSS, brugtmoms, rejsebureau (momsloven)</t>
         </is>
       </c>
-      <c r="I95" s="2" t="inlineStr">
+      <c r="K95" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat12_ecommerce_special.py</t>
         </is>
       </c>
-      <c r="J95" s="2" t="inlineStr">
+      <c r="L95" s="2" t="inlineStr">
         <is>
           <t>test_94_eu_b2c_oss</t>
         </is>
       </c>
-      <c r="K95" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L95" s="2" t="inlineStr"/>
+      <c r="M95" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N95" s="2" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -5942,25 +6896,35 @@
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
+          <t>E-handel &amp; særordninger</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
           <t>E-handel, digitale ydelser og særordninger: OSS, brugtmoms, rejsebureau (momsloven)</t>
         </is>
       </c>
-      <c r="I96" s="2" t="inlineStr">
+      <c r="K96" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat12_ecommerce_special.py</t>
         </is>
       </c>
-      <c r="J96" s="2" t="inlineStr">
+      <c r="L96" s="2" t="inlineStr">
         <is>
           <t>test_95_distance_selling_threshold</t>
         </is>
       </c>
-      <c r="K96" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L96" s="2" t="inlineStr"/>
+      <c r="M96" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N96" s="2" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -5998,25 +6962,35 @@
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
+          <t>E-handel &amp; særordninger</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
           <t>E-handel, digitale ydelser og særordninger: OSS, brugtmoms, rejsebureau (momsloven)</t>
         </is>
       </c>
-      <c r="I97" s="2" t="inlineStr">
+      <c r="K97" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat12_ecommerce_special.py</t>
         </is>
       </c>
-      <c r="J97" s="2" t="inlineStr">
+      <c r="L97" s="2" t="inlineStr">
         <is>
           <t>test_96_digital_service_eu_consumer</t>
         </is>
       </c>
-      <c r="K97" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L97" s="2" t="inlineStr"/>
+      <c r="M97" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N97" s="2" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -6054,25 +7028,35 @@
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
+          <t>E-handel &amp; særordninger</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
           <t>E-handel, digitale ydelser og særordninger: OSS, brugtmoms, rejsebureau (momsloven)</t>
         </is>
       </c>
-      <c r="I98" s="2" t="inlineStr">
+      <c r="K98" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat12_ecommerce_special.py</t>
         </is>
       </c>
-      <c r="J98" s="2" t="inlineStr">
+      <c r="L98" s="2" t="inlineStr">
         <is>
           <t>test_97_dk_vat_on_eu_consumer</t>
         </is>
       </c>
-      <c r="K98" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L98" s="2" t="inlineStr"/>
+      <c r="M98" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N98" s="2" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -6110,25 +7094,35 @@
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
+          <t>E-handel &amp; særordninger</t>
+        </is>
+      </c>
+      <c r="I99" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
           <t>E-handel, digitale ydelser og særordninger: OSS, brugtmoms, rejsebureau (momsloven)</t>
         </is>
       </c>
-      <c r="I99" s="2" t="inlineStr">
+      <c r="K99" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat12_ecommerce_special.py</t>
         </is>
       </c>
-      <c r="J99" s="2" t="inlineStr">
+      <c r="L99" s="2" t="inlineStr">
         <is>
           <t>test_98_ioss_low_value</t>
         </is>
       </c>
-      <c r="K99" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L99" s="2" t="inlineStr"/>
+      <c r="M99" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N99" s="2" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -6158,25 +7152,35 @@
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
+          <t>E-handel &amp; særordninger</t>
+        </is>
+      </c>
+      <c r="I100" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
           <t>E-handel, digitale ydelser og særordninger: OSS, brugtmoms, rejsebureau (momsloven)</t>
         </is>
       </c>
-      <c r="I100" s="2" t="inlineStr">
+      <c r="K100" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat12_ecommerce_special.py</t>
         </is>
       </c>
-      <c r="J100" s="2" t="inlineStr">
+      <c r="L100" s="2" t="inlineStr">
         <is>
           <t>test_99_platform_liability</t>
         </is>
       </c>
-      <c r="K100" s="2" t="inlineStr">
+      <c r="M100" s="2" t="inlineStr">
         <is>
           <t>(udfyldes — Fase C)</t>
         </is>
       </c>
-      <c r="L100" s="2" t="inlineStr">
+      <c r="N100" s="2" t="inlineStr">
         <is>
           <t>salgskanal + underliggende sælger (markedsplads-hæftelse)</t>
         </is>
@@ -6218,25 +7222,35 @@
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
+          <t>E-handel &amp; særordninger</t>
+        </is>
+      </c>
+      <c r="I101" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
           <t>E-handel, digitale ydelser og særordninger: OSS, brugtmoms, rejsebureau (momsloven)</t>
         </is>
       </c>
-      <c r="I101" s="2" t="inlineStr">
+      <c r="K101" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat12_ecommerce_special.py</t>
         </is>
       </c>
-      <c r="J101" s="2" t="inlineStr">
+      <c r="L101" s="2" t="inlineStr">
         <is>
           <t>test_100_electronic_services</t>
         </is>
       </c>
-      <c r="K101" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L101" s="2" t="inlineStr"/>
+      <c r="M101" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N101" s="2" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -6274,25 +7288,35 @@
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
+          <t>E-handel &amp; særordninger</t>
+        </is>
+      </c>
+      <c r="I102" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
           <t>E-handel, digitale ydelser og særordninger: OSS, brugtmoms, rejsebureau (momsloven)</t>
         </is>
       </c>
-      <c r="I102" s="2" t="inlineStr">
+      <c r="K102" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat12_ecommerce_special.py</t>
         </is>
       </c>
-      <c r="J102" s="2" t="inlineStr">
+      <c r="L102" s="2" t="inlineStr">
         <is>
           <t>test_101_telecom_broadcasting</t>
         </is>
       </c>
-      <c r="K102" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L102" s="2" t="inlineStr"/>
+      <c r="M102" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N102" s="2" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -6330,25 +7354,35 @@
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
+          <t>E-handel &amp; særordninger</t>
+        </is>
+      </c>
+      <c r="I103" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J103" s="2" t="inlineStr">
+        <is>
           <t>E-handel, digitale ydelser og særordninger: OSS, brugtmoms, rejsebureau (momsloven)</t>
         </is>
       </c>
-      <c r="I103" s="2" t="inlineStr">
+      <c r="K103" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat12_ecommerce_special.py</t>
         </is>
       </c>
-      <c r="J103" s="2" t="inlineStr">
+      <c r="L103" s="2" t="inlineStr">
         <is>
           <t>test_102_travel_margin</t>
         </is>
       </c>
-      <c r="K103" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L103" s="2" t="inlineStr"/>
+      <c r="M103" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N103" s="2" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -6386,33 +7420,217 @@
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
+          <t>E-handel &amp; særordninger</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="J104" s="2" t="inlineStr">
+        <is>
           <t>E-handel, digitale ydelser og særordninger: OSS, brugtmoms, rejsebureau (momsloven)</t>
         </is>
       </c>
-      <c r="I104" s="2" t="inlineStr">
+      <c r="K104" s="2" t="inlineStr">
         <is>
           <t>analytics/categories/cat12_ecommerce_special.py</t>
         </is>
       </c>
-      <c r="J104" s="2" t="inlineStr">
+      <c r="L104" s="2" t="inlineStr">
         <is>
           <t>test_103_used_goods_margin</t>
         </is>
       </c>
-      <c r="K104" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
-        </is>
-      </c>
-      <c r="L104" s="2" t="inlineStr"/>
+      <c r="M104" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_validation_suite.py + validation/scenarios.py</t>
+        </is>
+      </c>
+      <c r="N104" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:N1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Modul</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Nøgle</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Default</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Kontroller</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Beskrivelse</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Momskerne</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>moms_kerne</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>TIL</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Kontroller med direkte momsfaglig konsekvens: sats, fradragsret, angivelse, reverse charge, place-of-supply og momsafstemning. Fundamentet i en momsgennemgang.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Forensic &amp; statistik</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>forensic_statistik</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Statistisk anomalidetektion, beløbs-outliers, timing-anomalier og karrusel/MTIC-indikatorer. Hører til et JE-/besvigelsesmandat — ikke en momsgennemgang.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Stamdata- &amp; datakvalitet</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>datakvalitet</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Parts-/stamdatavalidering uden direkte fradrags-konsekvens (fx dubletnavne, formatfejl). Datakvalitet, ikke momsfund.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Dublet-recovery (bredt)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>dublet_recovery</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Bredere dublet-/recovery-scanninger (nær-dubletter, beløbsmatch på tværs). Den stærke eksakt-dublet med moms-dobbeltfradrag ligger i momskernen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>E-handel &amp; særordninger</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>ehandel_saerordninger</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>OSS/fjernsalg, digitale ydelser, margin-/brugtmoms. Momsfagligt korrekte, men kun relevante ved B2C-fjernsalg/særordninger — klientbetinget, default fra.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>